<commit_message>
added test cases; added test logs; cleaned-up some code
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{677DC8E8-422F-4DEE-A6B2-81373C481FBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\echan\IdeaProjects\selenium_prac\src\test\resources\testdata\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13B01678-61FD-4096-9D12-6A72D6EF44B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Geolocation_Tracking_Data" sheetId="6" r:id="rId1"/>
@@ -40,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="142">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -105,17 +110,6 @@
     <t>Year</t>
   </si>
   <si>
-    <t>RS-TC-005
-RS-TC-007
-RS-TC-011
-RS-TC-015
-RS-TC-019
-RS-TC-020
-RS-TC-022
-RS-TC-026
-RS-TC-030</t>
-  </si>
-  <si>
     <t>Jane</t>
   </si>
   <si>
@@ -137,36 +131,24 @@
     <t>Valid</t>
   </si>
   <si>
-    <t>RS-TC-004</t>
-  </si>
-  <si>
     <t>Jane123!</t>
   </si>
   <si>
     <t>Invalid First Name</t>
   </si>
   <si>
-    <t>RS-TC-006</t>
-  </si>
-  <si>
     <t>Doe123!</t>
   </si>
   <si>
     <t>Invalid Last Name</t>
   </si>
   <si>
-    <t>RS-TC-010</t>
-  </si>
-  <si>
     <t>janedoe.com</t>
   </si>
   <si>
     <t>Invalid Email</t>
   </si>
   <si>
-    <t>RS-TC-012</t>
-  </si>
-  <si>
     <t>testing!</t>
   </si>
   <si>
@@ -179,9 +161,6 @@
     <t>Invalid Phone Number Format</t>
   </si>
   <si>
-    <t>RS-TC-014</t>
-  </si>
-  <si>
     <t>RS-TC-016</t>
   </si>
   <si>
@@ -210,9 +189,6 @@
   </si>
   <si>
     <t>Invalid Confirm Password</t>
-  </si>
-  <si>
-    <t>RS-TC-031</t>
   </si>
   <si>
     <t>John</t>
@@ -463,12 +439,63 @@
   <si>
     <t>OS-TC-020</t>
   </si>
+  <si>
+    <t>RS-TC-005</t>
+  </si>
+  <si>
+    <t>RS-TC-008</t>
+  </si>
+  <si>
+    <t>091234567</t>
+  </si>
+  <si>
+    <t>RS-TC-022</t>
+  </si>
+  <si>
+    <t>RS-TC-023</t>
+  </si>
+  <si>
+    <t>RS-TC-026</t>
+  </si>
+  <si>
+    <t>RS-TC-030</t>
+  </si>
+  <si>
+    <t>Invalid Birthday (Future date)</t>
+  </si>
+  <si>
+    <t>RS-TC-011
+RS-TC-035</t>
+  </si>
+  <si>
+    <t>RS-TC-034</t>
+  </si>
+  <si>
+    <t>RS-TC-006
+RS-TC-009
+RS-TC-011
+RS-TC-014
+RS-TC-019
+RS-TC-024
+RS-TC-025
+RS-TC-027
+RS-TC-031</t>
+  </si>
+  <si>
+    <t>Invalid, Existing Email</t>
+  </si>
+  <si>
+    <t>Joshua</t>
+  </si>
+  <si>
+    <t>Cruz</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -606,9 +633,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -646,7 +673,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -752,7 +779,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -894,7 +921,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -903,14 +930,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00C45F4C-7522-4BA7-A3CA-2C78A83FEAFA}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.85546875" customWidth="1"/>
-    <col min="2" max="2" width="21.140625" customWidth="1"/>
-    <col min="3" max="3" width="17.85546875" customWidth="1"/>
+    <col min="1" max="1" width="11.81640625" customWidth="1"/>
+    <col min="2" max="2" width="21.1796875" customWidth="1"/>
+    <col min="3" max="3" width="17.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -921,7 +948,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>3</v>
       </c>
@@ -932,7 +959,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>6</v>
       </c>
@@ -943,7 +970,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>9</v>
       </c>
@@ -954,7 +981,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
         <v>10</v>
       </c>
@@ -972,19 +999,19 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L13"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:L16"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.85546875" customWidth="1"/>
-    <col min="2" max="2" width="10.42578125" customWidth="1"/>
-    <col min="3" max="4" width="11.42578125" customWidth="1"/>
+    <col min="1" max="1" width="12.81640625" customWidth="1"/>
+    <col min="2" max="2" width="10.453125" customWidth="1"/>
+    <col min="3" max="4" width="11.453125" customWidth="1"/>
     <col min="5" max="5" width="32" customWidth="1"/>
-    <col min="6" max="6" width="14.85546875" customWidth="1"/>
-    <col min="7" max="8" width="16.7109375" customWidth="1"/>
-    <col min="12" max="12" width="19.5703125" customWidth="1"/>
+    <col min="6" max="6" width="14.81640625" customWidth="1"/>
+    <col min="7" max="8" width="16.7265625" customWidth="1"/>
+    <col min="12" max="12" width="19.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1022,30 +1049,30 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="137.25">
+    <row r="2" spans="1:12" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="B2" t="s">
         <v>21</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>22</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>23</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>24</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="G2" t="s">
         <v>26</v>
       </c>
-      <c r="G2" t="s">
-        <v>27</v>
-      </c>
       <c r="H2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I2">
         <v>19</v>
@@ -1057,33 +1084,33 @@
         <v>2002</v>
       </c>
       <c r="L2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>128</v>
+      </c>
+      <c r="B3" s="7" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="3" spans="1:12">
-      <c r="A3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>30</v>
-      </c>
       <c r="C3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3" t="s">
         <v>23</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>24</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="G3" t="s">
         <v>26</v>
       </c>
-      <c r="G3" t="s">
-        <v>27</v>
-      </c>
       <c r="H3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I3">
         <v>19</v>
@@ -1095,33 +1122,33 @@
         <v>2002</v>
       </c>
       <c r="L3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>32</v>
+        <v>129</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" t="s">
         <v>24</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="G4" t="s">
         <v>26</v>
       </c>
-      <c r="G4" t="s">
-        <v>27</v>
-      </c>
       <c r="H4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I4">
         <v>19</v>
@@ -1133,33 +1160,33 @@
         <v>2002</v>
       </c>
       <c r="L4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" t="s">
         <v>22</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>23</v>
       </c>
-      <c r="D5" t="s">
-        <v>24</v>
-      </c>
       <c r="E5" s="8" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="F5" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" t="s">
         <v>26</v>
       </c>
-      <c r="G5" t="s">
-        <v>27</v>
-      </c>
       <c r="H5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I5">
         <v>19</v>
@@ -1171,33 +1198,33 @@
         <v>2002</v>
       </c>
       <c r="L5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>38</v>
       </c>
       <c r="B6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" t="s">
         <v>22</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>23</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>24</v>
       </c>
-      <c r="E6" t="s">
-        <v>25</v>
-      </c>
       <c r="F6" s="7" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="G6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I6">
         <v>19</v>
@@ -1209,33 +1236,33 @@
         <v>2002</v>
       </c>
       <c r="L6" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>41</v>
       </c>
       <c r="B7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" t="s">
         <v>22</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>23</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>24</v>
-      </c>
-      <c r="E7" t="s">
-        <v>25</v>
       </c>
       <c r="F7" s="9">
         <v>12345678900</v>
       </c>
       <c r="G7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I7">
         <v>19</v>
@@ -1247,33 +1274,33 @@
         <v>2002</v>
       </c>
       <c r="L7" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>43</v>
       </c>
       <c r="B8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" t="s">
         <v>22</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>23</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>24</v>
       </c>
-      <c r="E8" t="s">
-        <v>25</v>
-      </c>
-      <c r="F8" s="9">
-        <v>91234567</v>
+      <c r="F8" s="9" t="s">
+        <v>130</v>
       </c>
       <c r="G8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I8">
         <v>19</v>
@@ -1285,33 +1312,33 @@
         <v>2002</v>
       </c>
       <c r="L8" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B9" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" t="s">
         <v>22</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>23</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>24</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F9" s="5" t="s">
-        <v>26</v>
-      </c>
       <c r="G9" s="7" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="I9">
         <v>19</v>
@@ -1323,33 +1350,33 @@
         <v>2002</v>
       </c>
       <c r="L9" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>47</v>
+        <v>131</v>
       </c>
       <c r="B10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" t="s">
         <v>22</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>23</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>24</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F10" s="5" t="s">
-        <v>26</v>
-      </c>
       <c r="G10" s="8" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="I10">
         <v>19</v>
@@ -1361,33 +1388,33 @@
         <v>2002</v>
       </c>
       <c r="L10" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>49</v>
+        <v>132</v>
       </c>
       <c r="B11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" t="s">
         <v>22</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>23</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>24</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F11" s="5" t="s">
-        <v>26</v>
-      </c>
       <c r="G11" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="H11" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="I11">
         <v>19</v>
@@ -1399,30 +1426,30 @@
         <v>2002</v>
       </c>
       <c r="L11" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>52</v>
+        <v>133</v>
       </c>
       <c r="B12" t="s">
+        <v>21</v>
+      </c>
+      <c r="C12" t="s">
         <v>22</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>23</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>24</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F12" s="5" t="s">
+      <c r="G12" t="s">
         <v>26</v>
-      </c>
-      <c r="G12" t="s">
-        <v>27</v>
       </c>
       <c r="H12" s="7" t="s">
         <v>16</v>
@@ -1437,46 +1464,126 @@
         <v>2002</v>
       </c>
       <c r="L12" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12">
-      <c r="A13" t="s">
-        <v>54</v>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A13" s="6" t="s">
+        <v>134</v>
       </c>
       <c r="B13" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="C13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D13" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="E13" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="G13" t="s">
+        <v>26</v>
+      </c>
+      <c r="H13" t="s">
+        <v>26</v>
+      </c>
+      <c r="I13" s="7">
+        <v>31</v>
+      </c>
+      <c r="J13" s="7">
+        <v>12</v>
+      </c>
+      <c r="K13" s="7">
+        <v>2026</v>
+      </c>
+      <c r="L13" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>137</v>
+      </c>
+      <c r="B14" t="s">
+        <v>140</v>
+      </c>
+      <c r="C14" t="s">
+        <v>141</v>
+      </c>
+      <c r="D14" t="s">
+        <v>49</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G14" t="s">
+        <v>26</v>
+      </c>
+      <c r="H14" t="s">
+        <v>26</v>
+      </c>
+      <c r="I14">
+        <v>19</v>
+      </c>
+      <c r="J14">
+        <v>9</v>
+      </c>
+      <c r="K14">
+        <v>2002</v>
+      </c>
+      <c r="L14" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+      <c r="A15" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="B15" t="s">
+        <v>48</v>
+      </c>
+      <c r="C15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D15" t="s">
+        <v>49</v>
+      </c>
+      <c r="E15" t="s">
+        <v>50</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="G15" t="s">
+        <v>26</v>
+      </c>
+      <c r="H15" t="s">
+        <v>26</v>
+      </c>
+      <c r="I15">
+        <v>19</v>
+      </c>
+      <c r="J15">
+        <v>9</v>
+      </c>
+      <c r="K15">
+        <v>2002</v>
+      </c>
+      <c r="L15" t="s">
         <v>27</v>
       </c>
-      <c r="H13" t="s">
-        <v>27</v>
-      </c>
-      <c r="I13">
-        <v>19</v>
-      </c>
-      <c r="J13">
-        <v>9</v>
-      </c>
-      <c r="K13">
-        <v>2002</v>
-      </c>
-      <c r="L13" t="s">
-        <v>28</v>
-      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A16" s="6"/>
+      <c r="F16" s="2"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1498,18 +1605,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F68DF73-E7CD-4240-9557-2AA4119DA34C}">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" customWidth="1"/>
-    <col min="2" max="2" width="21.7109375" customWidth="1"/>
-    <col min="3" max="3" width="15.140625" customWidth="1"/>
-    <col min="4" max="4" width="21.5703125" customWidth="1"/>
+    <col min="1" max="1" width="11.7265625" customWidth="1"/>
+    <col min="2" max="2" width="21.7265625" customWidth="1"/>
+    <col min="3" max="3" width="15.1796875" customWidth="1"/>
+    <col min="4" max="4" width="21.54296875" customWidth="1"/>
     <col min="5" max="5" width="32" customWidth="1"/>
-    <col min="6" max="6" width="14.85546875" customWidth="1"/>
-    <col min="7" max="8" width="16.7109375" customWidth="1"/>
+    <col min="6" max="6" width="14.81640625" customWidth="1"/>
+    <col min="7" max="8" width="16.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1523,39 +1630,39 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="30.75">
+    <row r="2" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="D2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="30.75">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="D3" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="F3" s="5"/>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="F4" s="5"/>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="F5" s="5"/>
     </row>
   </sheetData>
@@ -1566,15 +1673,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC4C55B6-D732-476E-AEB9-DF4442E1A12D}">
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="30.28515625" customWidth="1"/>
-    <col min="3" max="3" width="16.140625" customWidth="1"/>
-    <col min="4" max="4" width="22.5703125" customWidth="1"/>
+    <col min="2" max="2" width="30.26953125" customWidth="1"/>
+    <col min="3" max="3" width="16.1796875" customWidth="1"/>
+    <col min="4" max="4" width="22.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1588,74 +1695,74 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="D3" t="s">
         <v>66</v>
       </c>
-      <c r="B2" s="3" t="s">
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>67</v>
       </c>
-      <c r="C2" t="s">
+      <c r="B4" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="D2" t="s">
+      <c r="C4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" t="s">
+      <c r="B5" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="D5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>70</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B6" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C6" t="s">
         <v>71</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="D6" s="6" t="s">
         <v>72</v>
-      </c>
-      <c r="D3" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
-        <v>74</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="C4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D4" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" t="s">
-        <v>76</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="D5" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="30.75">
-      <c r="A6" t="s">
-        <v>77</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="C6" t="s">
-        <v>78</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -1666,15 +1773,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9EA7360-13D0-453E-8437-7172C5B81D7D}">
   <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.28515625" customWidth="1"/>
-    <col min="2" max="2" width="29.42578125" customWidth="1"/>
+    <col min="1" max="1" width="16.26953125" customWidth="1"/>
+    <col min="2" max="2" width="29.453125" customWidth="1"/>
     <col min="3" max="4" width="22" customWidth="1"/>
-    <col min="5" max="5" width="22.28515625" customWidth="1"/>
+    <col min="5" max="5" width="22.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1685,84 +1792,84 @@
         <v>16</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="C2" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="D2" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="E2" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="C3" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="D3" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="E3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="E4" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="C5" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="E5" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B6" s="3"/>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="3"/>
     </row>
   </sheetData>
@@ -1773,33 +1880,33 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA628117-8171-40AF-9E76-62A43F156754}">
   <dimension ref="A1:M13"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.85546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.7109375" style="6" customWidth="1"/>
+    <col min="1" max="1" width="11.81640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.7265625" style="6" customWidth="1"/>
     <col min="3" max="3" width="10" style="6" customWidth="1"/>
-    <col min="4" max="4" width="10.85546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.85546875" style="6" customWidth="1"/>
-    <col min="7" max="7" width="23.140625" style="6" customWidth="1"/>
-    <col min="8" max="8" width="15.7109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="34.28515625" style="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.42578125" style="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="32.28515625" style="6" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="7.7109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.42578125" style="6" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="9.140625" style="6"/>
+    <col min="4" max="4" width="10.81640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.453125" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.81640625" style="6" customWidth="1"/>
+    <col min="7" max="7" width="23.1796875" style="6" customWidth="1"/>
+    <col min="8" max="8" width="15.7265625" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="34.26953125" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.453125" style="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="32.26953125" style="6" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.7265625" style="6" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.453125" style="6" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="9.1796875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>11</v>
@@ -1808,54 +1915,54 @@
         <v>12</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="G1" s="10" t="s">
         <v>14</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="J1" s="10" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="K1" s="11" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="L1" s="10" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="M1" s="10" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="91.5">
+    <row r="2" spans="1:13" ht="87" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="F2" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="H2" s="6" t="s">
         <v>96</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="C2" s="12" t="s">
-        <v>98</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="F2" s="12" t="s">
-        <v>101</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="H2" s="6" t="s">
-        <v>103</v>
       </c>
       <c r="I2" s="6">
         <v>1212</v>
@@ -1864,39 +1971,39 @@
         <v>123</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="L2" s="6">
         <v>1000</v>
       </c>
       <c r="M2" s="6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" ht="30.75">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="F3" s="6">
         <v>12345678912</v>
       </c>
       <c r="G3" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="I3" s="6">
         <v>1212</v>
@@ -1905,39 +2012,39 @@
         <v>123</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="L3" s="6">
         <v>1000</v>
       </c>
       <c r="M3" s="6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" ht="30.75">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="E4" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="F4" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="F4" s="12" t="s">
-        <v>107</v>
-      </c>
       <c r="G4" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="I4" s="6">
         <v>1212</v>
@@ -1946,39 +2053,39 @@
         <v>123</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="L4" s="6">
         <v>1000</v>
       </c>
       <c r="M4" s="6" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="I5" s="6">
         <v>1212</v>
@@ -1987,39 +2094,39 @@
         <v>123</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="L5" s="6">
         <v>1000</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="I6" s="6">
         <v>1212</v>
@@ -2028,36 +2135,36 @@
         <v>123</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="L6" s="6">
         <v>10</v>
       </c>
       <c r="M6" s="6" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="F7" s="14"/>
     </row>
-    <row r="8" spans="1:13">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="F8" s="14"/>
     </row>
-    <row r="9" spans="1:13">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="F9" s="12"/>
     </row>
-    <row r="10" spans="1:13">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="F10" s="12"/>
       <c r="G10" s="13"/>
       <c r="H10" s="13"/>
     </row>
-    <row r="11" spans="1:13">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="F11" s="12"/>
     </row>
-    <row r="12" spans="1:13">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="F12" s="12"/>
     </row>
-    <row r="13" spans="1:13">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="F13" s="15"/>
     </row>
   </sheetData>
@@ -2068,25 +2175,25 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{237319F2-5C9C-4AF4-8EFE-3242F7D6CB15}">
   <dimension ref="A1:L11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14" style="6" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="6" customWidth="1"/>
-    <col min="3" max="3" width="22.85546875" style="6" customWidth="1"/>
-    <col min="4" max="4" width="13.85546875" style="6" customWidth="1"/>
-    <col min="5" max="5" width="14.140625" style="6" customWidth="1"/>
-    <col min="6" max="6" width="11.42578125" style="6" customWidth="1"/>
-    <col min="7" max="10" width="9.140625" style="6"/>
-    <col min="11" max="11" width="11.7109375" style="6" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="6"/>
+    <col min="2" max="2" width="30.453125" style="6" customWidth="1"/>
+    <col min="3" max="3" width="22.81640625" style="6" customWidth="1"/>
+    <col min="4" max="4" width="13.81640625" style="6" customWidth="1"/>
+    <col min="5" max="5" width="14.1796875" style="6" customWidth="1"/>
+    <col min="6" max="6" width="11.453125" style="6" customWidth="1"/>
+    <col min="7" max="10" width="9.1796875" style="6"/>
+    <col min="11" max="11" width="11.7265625" style="6" customWidth="1"/>
+    <col min="12" max="16384" width="9.1796875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>2</v>
@@ -2101,118 +2208,118 @@
       <c r="K1" s="10"/>
       <c r="L1" s="10"/>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" ht="30.75">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" s="10" t="s">
         <v>0</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A7" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="17" t="s">
+        <v>121</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+      <c r="A9" s="17" t="s">
         <v>123</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B9" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="D9" s="6" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="7" spans="1:12">
-      <c r="A7" s="13" t="s">
+      <c r="E9" s="6" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A10" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B10" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+      <c r="A11" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="B11" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="D11" s="13" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" ht="76.5">
-      <c r="A8" s="17" t="s">
-        <v>128</v>
-      </c>
-      <c r="B8" s="13" t="s">
-        <v>127</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" ht="30.75">
-      <c r="A9" s="17" t="s">
-        <v>130</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12">
-      <c r="A10" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" ht="30.75">
-      <c r="A11" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="D11" s="13" t="s">
-        <v>132</v>
-      </c>
       <c r="E11" s="6" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
more register test cases changes and optimizations
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\echan\IdeaProjects\selenium_prac\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13B01678-61FD-4096-9D12-6A72D6EF44B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96A2800C-BD31-42B6-8F30-CB57CD71F0DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Geolocation_Tracking_Data" sheetId="6" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="141">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -262,17 +262,11 @@
     <t>LS-TC-013</t>
   </si>
   <si>
-    <t xml:space="preserve">Password@1234 </t>
-  </si>
-  <si>
     <t>Pre:Requisite: LS-TC-009
 Valid Updated Password</t>
   </si>
   <si>
     <t>Confirm Password</t>
-  </si>
-  <si>
-    <t>LS-TC-012</t>
   </si>
   <si>
     <t>Valid Password Update</t>
@@ -464,31 +458,40 @@
     <t>Invalid Birthday (Future date)</t>
   </si>
   <si>
-    <t>RS-TC-011
+    <t>RS-TC-034</t>
+  </si>
+  <si>
+    <t>Invalid, Existing Email</t>
+  </si>
+  <si>
+    <t>Joshua</t>
+  </si>
+  <si>
+    <t>Cruz</t>
+  </si>
+  <si>
+    <t>RS-TC-011 
 RS-TC-035</t>
   </si>
   <si>
-    <t>RS-TC-034</t>
-  </si>
-  <si>
-    <t>RS-TC-006
+    <t>LS-TC-014</t>
+  </si>
+  <si>
+    <t>RS-TC-004
+RS-TC-006
+RS-TC-007
 RS-TC-009
 RS-TC-011
+RS-TC-012
 RS-TC-014
+RS-TC-015
 RS-TC-019
+RS-TC-020
 RS-TC-024
 RS-TC-025
 RS-TC-027
-RS-TC-031</t>
-  </si>
-  <si>
-    <t>Invalid, Existing Email</t>
-  </si>
-  <si>
-    <t>Joshua</t>
-  </si>
-  <si>
-    <t>Cruz</t>
+RS-TC-031
+RS-TC-033</t>
   </si>
 </sst>
 </file>
@@ -1049,9 +1052,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B2" t="s">
         <v>21</v>
@@ -1089,7 +1092,7 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>28</v>
@@ -1127,7 +1130,7 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B4" t="s">
         <v>21</v>
@@ -1294,7 +1297,7 @@
         <v>24</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="G8" t="s">
         <v>26</v>
@@ -1320,16 +1323,16 @@
         <v>46</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
+        <v>48</v>
       </c>
       <c r="C9" t="s">
         <v>22</v>
       </c>
       <c r="D9" t="s">
-        <v>23</v>
+        <v>49</v>
       </c>
       <c r="E9" t="s">
-        <v>24</v>
+        <v>50</v>
       </c>
       <c r="F9" s="5" t="s">
         <v>25</v>
@@ -1355,19 +1358,19 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B10" t="s">
-        <v>21</v>
+        <v>48</v>
       </c>
       <c r="C10" t="s">
         <v>22</v>
       </c>
       <c r="D10" t="s">
-        <v>23</v>
+        <v>49</v>
       </c>
       <c r="E10" t="s">
-        <v>24</v>
+        <v>50</v>
       </c>
       <c r="F10" s="5" t="s">
         <v>25</v>
@@ -1393,7 +1396,7 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B11" t="s">
         <v>21</v>
@@ -1431,7 +1434,7 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B12" t="s">
         <v>21</v>
@@ -1469,7 +1472,7 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13" s="6" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B13" t="s">
         <v>48</v>
@@ -1502,18 +1505,18 @@
         <v>2026</v>
       </c>
       <c r="L13" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
+        <v>134</v>
+      </c>
+      <c r="B14" t="s">
+        <v>136</v>
+      </c>
+      <c r="C14" t="s">
         <v>137</v>
-      </c>
-      <c r="B14" t="s">
-        <v>140</v>
-      </c>
-      <c r="C14" t="s">
-        <v>141</v>
       </c>
       <c r="D14" t="s">
         <v>49</v>
@@ -1540,12 +1543,12 @@
         <v>2002</v>
       </c>
       <c r="L14" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B15" t="s">
         <v>48</v>
@@ -1587,16 +1590,14 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1" xr:uid="{CCE1B043-06CC-4013-9A76-E0E181BD7292}"/>
-    <hyperlink ref="E3" r:id="rId2" xr:uid="{25906D00-026C-4E5B-A4C4-043FC917215A}"/>
-    <hyperlink ref="E4" r:id="rId3" xr:uid="{4D3EFBC2-78D8-43F5-9BFE-3F3DF10E822D}"/>
-    <hyperlink ref="E6" r:id="rId4" xr:uid="{C1FBCC98-E01D-4D79-8CF2-01A4C5E17F4E}"/>
-    <hyperlink ref="E7" r:id="rId5" xr:uid="{84243ED9-8659-43D8-89F3-60D073EF74DF}"/>
-    <hyperlink ref="E8" r:id="rId6" xr:uid="{304D0317-8016-4EC5-954B-881569CE5577}"/>
-    <hyperlink ref="E9" r:id="rId7" xr:uid="{21831FE6-9910-4DA2-8DCA-1D191425D61D}"/>
-    <hyperlink ref="E10" r:id="rId8" xr:uid="{19C94D56-C143-4371-B0C9-553BCAF9563A}"/>
-    <hyperlink ref="E11" r:id="rId9" xr:uid="{6EA55E52-C67F-498D-B89D-28F9B131C14C}"/>
-    <hyperlink ref="E12" r:id="rId10" xr:uid="{6CA94468-1FE5-4246-AF55-B1C81FAE2103}"/>
+    <hyperlink ref="E3" r:id="rId1" xr:uid="{25906D00-026C-4E5B-A4C4-043FC917215A}"/>
+    <hyperlink ref="E4" r:id="rId2" xr:uid="{4D3EFBC2-78D8-43F5-9BFE-3F3DF10E822D}"/>
+    <hyperlink ref="E6" r:id="rId3" xr:uid="{C1FBCC98-E01D-4D79-8CF2-01A4C5E17F4E}"/>
+    <hyperlink ref="E7" r:id="rId4" xr:uid="{84243ED9-8659-43D8-89F3-60D073EF74DF}"/>
+    <hyperlink ref="E8" r:id="rId5" xr:uid="{304D0317-8016-4EC5-954B-881569CE5577}"/>
+    <hyperlink ref="E11" r:id="rId6" xr:uid="{6EA55E52-C67F-498D-B89D-28F9B131C14C}"/>
+    <hyperlink ref="E12" r:id="rId7" xr:uid="{6CA94468-1FE5-4246-AF55-B1C81FAE2103}"/>
+    <hyperlink ref="E2" r:id="rId8" xr:uid="{CCE1B043-06CC-4013-9A76-E0E181BD7292}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1753,16 +1754,16 @@
     </row>
     <row r="6" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>70</v>
+        <v>139</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>60</v>
       </c>
       <c r="C6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" s="6" t="s">
         <v>71</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -1792,7 +1793,7 @@
         <v>16</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>2</v>
@@ -1800,7 +1801,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>60</v>
@@ -1812,12 +1813,12 @@
         <v>54</v>
       </c>
       <c r="E2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B3" s="8" t="s">
         <v>68</v>
@@ -1834,16 +1835,16 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>60</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E4" t="s">
         <v>40</v>
@@ -1851,7 +1852,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>60</v>
@@ -1860,7 +1861,7 @@
         <v>54</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E5" t="s">
         <v>47</v>
@@ -1903,10 +1904,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>11</v>
@@ -1915,25 +1916,25 @@
         <v>12</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G1" s="10" t="s">
         <v>14</v>
       </c>
       <c r="H1" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="J1" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="I1" s="10" t="s">
+      <c r="K1" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="J1" s="10" t="s">
+      <c r="L1" s="10" t="s">
         <v>86</v>
-      </c>
-      <c r="K1" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="L1" s="10" t="s">
-        <v>88</v>
       </c>
       <c r="M1" s="10" t="s">
         <v>2</v>
@@ -1941,28 +1942,28 @@
     </row>
     <row r="2" spans="1:13" ht="87" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C2" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="D2" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="E2" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="F2" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="G2" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="H2" s="6" t="s">
         <v>94</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="H2" s="6" t="s">
-        <v>96</v>
       </c>
       <c r="I2" s="6">
         <v>1212</v>
@@ -1971,7 +1972,7 @@
         <v>123</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="L2" s="6">
         <v>1000</v>
@@ -1982,28 +1983,28 @@
     </row>
     <row r="3" spans="1:13" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="D3" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="E3" s="6" t="s">
         <v>91</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>93</v>
       </c>
       <c r="F3" s="6">
         <v>12345678912</v>
       </c>
       <c r="G3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="I3" s="6">
         <v>1212</v>
@@ -2012,7 +2013,7 @@
         <v>123</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="L3" s="6">
         <v>1000</v>
@@ -2023,28 +2024,28 @@
     </row>
     <row r="4" spans="1:13" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="D4" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="E4" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="D4" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="E4" s="6" t="s">
+      <c r="F4" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="G4" t="s">
         <v>93</v>
       </c>
-      <c r="F4" s="12" t="s">
-        <v>100</v>
-      </c>
-      <c r="G4" t="s">
-        <v>95</v>
-      </c>
       <c r="H4" s="6" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="I4" s="6">
         <v>1212</v>
@@ -2053,39 +2054,39 @@
         <v>123</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="L4" s="6">
         <v>1000</v>
       </c>
       <c r="M4" s="6" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="E5" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="F5" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="E5" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="F5" s="12" t="s">
+      <c r="G5" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="H5" s="6" t="s">
         <v>94</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>96</v>
       </c>
       <c r="I5" s="6">
         <v>1212</v>
@@ -2094,7 +2095,7 @@
         <v>123</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="L5" s="6">
         <v>1000</v>
@@ -2105,28 +2106,28 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B6" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="D6" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="E6" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="F6" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="G6" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="F6" s="12" t="s">
+      <c r="H6" s="6" t="s">
         <v>94</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>96</v>
       </c>
       <c r="I6" s="6">
         <v>1212</v>
@@ -2135,13 +2136,13 @@
         <v>123</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="L6" s="6">
         <v>10</v>
       </c>
       <c r="M6" s="6" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.35">
@@ -2193,7 +2194,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>2</v>
@@ -2210,24 +2211,24 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C2" s="6" t="s">
         <v>107</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="C3" s="6" t="s">
         <v>110</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
@@ -2235,13 +2236,13 @@
         <v>0</v>
       </c>
       <c r="B5" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="D5" s="10" t="s">
         <v>113</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>114</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>115</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>2</v>
@@ -2249,77 +2250,77 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>116</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" s="13" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A8" s="17" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B8" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="C8" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="C8" s="6" t="s">
-        <v>122</v>
-      </c>
       <c r="E8" s="6" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="17" t="s">
+        <v>121</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="D9" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>125</v>
-      </c>
       <c r="E9" s="6" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>